<commit_message>
Record hosted #17 operational UX evidence for Product Leadership final review.
Vendor, deletion, consent, incident, import, and 12-slide board artifacts are from live staging SHA 9976e81. #17 remains PARTIAL.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/private-beta/hosted-ux-qa/supreme-privacy/Supreme-Privacy-Register.xlsx
+++ b/docs/private-beta/hosted-ux-qa/supreme-privacy/Supreme-Privacy-Register.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="26">
   <si>
     <t>ID</t>
   </si>
@@ -34,7 +34,7 @@
     <t>Claims servicing</t>
   </si>
   <si>
-    <t>ACTIVE</t>
+    <t>Active</t>
   </si>
   <si>
     <t>Report Proof</t>
@@ -43,30 +43,39 @@
     <t>PA-00002</t>
   </si>
   <si>
+    <t>PA-00003</t>
+  </si>
+  <si>
     <t>XFR-00001</t>
   </si>
   <si>
     <t>US-NY → IE</t>
   </si>
   <si>
-    <t>REVIEW REQUIRED</t>
+    <t>Review Required</t>
   </si>
   <si>
     <t>XFR-00002</t>
   </si>
   <si>
+    <t>XFR-00003</t>
+  </si>
+  <si>
     <t>DSR-00001</t>
   </si>
   <si>
-    <t>ACCESS</t>
-  </si>
-  <si>
-    <t>RECEIVED</t>
+    <t>Access</t>
+  </si>
+  <si>
+    <t>Received</t>
   </si>
   <si>
     <t>DSR-00002</t>
   </si>
   <si>
+    <t>DSR-00003</t>
+  </si>
+  <si>
     <t>RET-00001</t>
   </si>
   <si>
@@ -80,6 +89,9 @@
   </si>
   <si>
     <t>RET-00002</t>
+  </si>
+  <si>
+    <t>RET-00003</t>
   </si>
 </sst>
 </file>
@@ -456,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -498,6 +510,20 @@
         <v>6</v>
       </c>
       <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -509,7 +535,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -528,13 +554,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -542,15 +568,29 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -562,7 +602,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -581,13 +621,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -595,15 +635,29 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -615,7 +669,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -634,30 +688,44 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
         <v>21</v>
       </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record hosted #17 native Board PPTX and mobile deletion/incident evidence.
PowerPoint rendered the live Elite Claims deck; 375/768 cards keep primary privacy fields readable. Status stays PARTIAL for Product Leadership.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/private-beta/hosted-ux-qa/supreme-privacy/Supreme-Privacy-Register.xlsx
+++ b/docs/private-beta/hosted-ux-qa/supreme-privacy/Supreme-Privacy-Register.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
@@ -46,6 +46,9 @@
     <t>PA-00003</t>
   </si>
   <si>
+    <t>PA-00004</t>
+  </si>
+  <si>
     <t>XFR-00001</t>
   </si>
   <si>
@@ -61,6 +64,9 @@
     <t>XFR-00003</t>
   </si>
   <si>
+    <t>XFR-00004</t>
+  </si>
+  <si>
     <t>DSR-00001</t>
   </si>
   <si>
@@ -76,6 +82,9 @@
     <t>DSR-00003</t>
   </si>
   <si>
+    <t>DSR-00004</t>
+  </si>
+  <si>
     <t>RET-00001</t>
   </si>
   <si>
@@ -92,6 +101,9 @@
   </si>
   <si>
     <t>RET-00003</t>
+  </si>
+  <si>
+    <t>RET-00004</t>
   </si>
 </sst>
 </file>
@@ -468,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -524,6 +536,20 @@
         <v>6</v>
       </c>
       <c r="D4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -535,7 +561,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -554,13 +580,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -568,13 +594,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
         <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
@@ -582,15 +608,29 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="D4" t="s">
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -602,7 +642,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -621,13 +661,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -635,13 +675,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
         <v>18</v>
       </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
@@ -649,15 +689,29 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
         <v>19</v>
       </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
       <c r="D4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -669,7 +723,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -688,44 +742,58 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" t="s">
-        <v>21</v>
-      </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" t="s">
-        <v>22</v>
-      </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>